<commit_message>
Import Excel: per-row TyGiaUSD/VAT columns + auto suggested price (cost after VAT + 35%)
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -398,20 +398,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:N5"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
     <col min="9" max="9" width="14.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="46.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,9 +448,15 @@
         <v>GiaUSD</v>
       </c>
       <c r="K1" t="str">
+        <v>TyGiaUSD</v>
+      </c>
+      <c r="L1" t="str">
+        <v>VAT</v>
+      </c>
+      <c r="M1" t="str">
         <v>GiaBanDeXuat</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>GhiChu</v>
       </c>
     </row>
@@ -484,9 +492,15 @@
         <v>100</v>
       </c>
       <c r="K2">
+        <v>27000</v>
+      </c>
+      <c r="L2">
+        <v>8</v>
+      </c>
+      <c r="M2">
         <v>3936600</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>Dòng ví dụ — xoá trước khi dùng thật</v>
       </c>
     </row>
@@ -522,9 +536,15 @@
         <v>3.88</v>
       </c>
       <c r="K3">
+        <v>27000</v>
+      </c>
+      <c r="L3">
+        <v>8</v>
+      </c>
+      <c r="M3">
         <v>152740</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>Dòng ví dụ — xoá trước khi dùng thật</v>
       </c>
     </row>
@@ -560,24 +580,74 @@
         <v>3</v>
       </c>
       <c r="K4">
+        <v>27000</v>
+      </c>
+      <c r="L4">
+        <v>8</v>
+      </c>
+      <c r="M4">
         <v>118098</v>
       </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
         <v>Ví dụ nhiều mã thay thế cách nhau bằng '; '</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>VD-MINH-HOA</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>Ví dụ: để trống tỷ giá/VAT/giá bán</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>SMS</v>
+      </c>
+      <c r="F5" t="str">
+        <v>HOWO 420</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Cái</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5">
+        <v>10</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v>Để trống TyGiaUSD/VAT = dùng tỷ giá &amp; VAT trên form (vd 27.000 &amp; 8% → giá vốn 291.600); để trống Giá bán đề xuất = tự tính bằng giá vốn sau VAT + 35% (→ 393.660). Dòng ví dụ — xoá trước khi dùng thật</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A33"/>
   <cols>
-    <col min="1" max="1" width="150.83203125" customWidth="1"/>
+    <col min="1" max="1" width="130.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,12 +672,12 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Trong app TVK: vào 'Nhập từ Excel', chọn loại phiếu (Nhập mua / Nhập ký gửi), nhà cung cấp, kho, ngày — rồi tải file lên.</v>
+        <v>2. Trong app TVK: vào 'Nhập từ Excel', chọn loại phiếu (Nhập mua / Nhập ký gửi), nhà cung cấp, kho, ngày, tỷ giá và VAT mặc định — rồi tải file lên.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
+        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) kèm giá vốn, tỷ giá·VAT áp dụng, thành tiền và giá bán đề xuất — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
       </c>
     </row>
     <row r="7">
@@ -657,52 +727,97 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">   hệ thống tự tính Giá vốn = GiaUSD x Tỷ giá x (1 + VAT%) — tỷ giá và VAT% nhập trên form trong app (mặc định 27.000 và 8%).</v>
+        <v xml:space="preserve">   hệ thống tự tính Giá vốn = GiaUSD x Tỷ giá x (1 + VAT%) — xem mục CÔNG THỨC bên dưới.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GiaBanDeXuat: giá bán gợi ý — với hàng mới, hệ thống lưu thành giá bán buôn mặc định của sản phẩm.</v>
+        <v>TyGiaUSD (tuỳ chọn, theo từng dòng): tỷ giá VNĐ/USD riêng của dòng. Để trống = dùng tỷ giá trên form trong app.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GhiChu: ghi chú tự do cho dòng hàng.</v>
+        <v>VAT (tuỳ chọn, theo từng dòng, tính theo %): vd 8 = 8%. Để trống = dùng VAT trên form trong app. VAT = 0 nghĩa là không cộng VAT.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>GiaBanDeXuat: giá bán gợi ý — với hàng mới, hệ thống lưu thành giá bán buôn mặc định của sản phẩm. Để trống = tự tính (xem CÔNG THỨC).</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>LƯU Ý</v>
+        <v>GhiChu: ghi chú tự do cho dòng hàng.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>- Dòng thiếu MaHang hoặc SoLuong &lt;= 0 sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
+        <v>CÔNG THỨC (áp dụng cho mọi dòng)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm mã thay thế và dòng xe khi bạn xác nhận.</v>
+        <v>1. Giá vốn một đơn vị = GiaVonVND nếu có; ngược lại = GiaUSD x Tỷ giá x (1 + VAT%).</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>2. Tỷ giá và VAT lấy theo DÒNG (cột TyGiaUSD / VAT) nếu dòng có ghi; dòng nào để trống thì lấy tỷ giá và VAT trên form trong app (mặc định 27.000 và 8%).</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>3. Thành tiền của dòng = SoLuong x Giá vốn.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>4. Giá bán đề xuất = GiaBanDeXuat nếu có; để trống thì = Giá vốn sau VAT x 1,35 (tức giá vốn + 35%).</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>LƯU Ý</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>- Dòng thiếu MaHang hoặc SoLuong &lt;= 0 sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>- Dòng có TyGiaUSD &lt;= 0 hoặc VAT &lt; 0 cũng bị báo lỗi.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm mã thay thế và dòng xe khi bạn xác nhận.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
         <v>- Chấp nhận file .xlsx và .csv (csv: dùng đúng các tiêu đề cột như trên, mã hoá UTF-8).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Import Excel: 7-column input, form-level rate/VAT/profit applied to whole file
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -398,254 +398,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:G4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="8.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>DongXe</v>
+      </c>
+      <c r="B1" t="str">
+        <v>TenHang</v>
+      </c>
+      <c r="C1" t="str">
         <v>MaHang</v>
       </c>
-      <c r="B1" t="str">
-        <v>MaThayThe</v>
-      </c>
-      <c r="C1" t="str">
-        <v>TenHang</v>
-      </c>
       <c r="D1" t="str">
-        <v>TenTiengAnh</v>
+        <v>ThuongHieu</v>
       </c>
       <c r="E1" t="str">
-        <v>ThuongHieu</v>
+        <v>DonViTinh</v>
       </c>
       <c r="F1" t="str">
-        <v>DongXe</v>
+        <v>SoLuong</v>
       </c>
       <c r="G1" t="str">
-        <v>DonViTinh</v>
-      </c>
-      <c r="H1" t="str">
-        <v>SoLuong</v>
-      </c>
-      <c r="I1" t="str">
-        <v>GiaVonVND</v>
-      </c>
-      <c r="J1" t="str">
         <v>GiaUSD</v>
-      </c>
-      <c r="K1" t="str">
-        <v>TyGiaUSD</v>
-      </c>
-      <c r="L1" t="str">
-        <v>VAT</v>
-      </c>
-      <c r="M1" t="str">
-        <v>GiaBanDeXuat</v>
-      </c>
-      <c r="N1" t="str">
-        <v>GhiChu</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>HOWO 420</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Bơm nước - 420Hp</v>
+      </c>
+      <c r="C2" t="str">
         <v>VG1246060108</v>
       </c>
-      <c r="B2" t="str">
-        <v>SMS-10636</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Bơm nước - 420Hp</v>
-      </c>
       <c r="D2" t="str">
-        <v>Water Pump - 420Hp</v>
+        <v>SMS</v>
       </c>
       <c r="E2" t="str">
-        <v>SMS</v>
-      </c>
-      <c r="F2" t="str">
-        <v>HOWO 420</v>
-      </c>
-      <c r="G2" t="str">
         <v>Cái</v>
       </c>
-      <c r="H2">
+      <c r="F2">
         <v>15</v>
       </c>
-      <c r="I2">
-        <v>2916000</v>
-      </c>
-      <c r="J2">
+      <c r="G2">
         <v>100</v>
-      </c>
-      <c r="K2">
-        <v>27000</v>
-      </c>
-      <c r="L2">
-        <v>8</v>
-      </c>
-      <c r="M2">
-        <v>3936600</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Dòng ví dụ — xoá trước khi dùng thật</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>HOWO 430</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Lọc dầu dưới</v>
+      </c>
+      <c r="C3" t="str">
         <v>611600080113</v>
       </c>
-      <c r="B3" t="str">
-        <v>1001362240</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Lọc dầu dưới</v>
-      </c>
       <c r="D3" t="str">
-        <v>Fuel Filter</v>
+        <v>SMS</v>
       </c>
       <c r="E3" t="str">
-        <v>SMS</v>
-      </c>
-      <c r="F3" t="str">
-        <v>HOWO 430</v>
-      </c>
-      <c r="G3" t="str">
         <v>Cái</v>
       </c>
-      <c r="H3">
+      <c r="F3">
         <v>400</v>
       </c>
-      <c r="I3">
-        <v>113141</v>
-      </c>
-      <c r="J3">
+      <c r="G3">
         <v>3.88</v>
-      </c>
-      <c r="K3">
-        <v>27000</v>
-      </c>
-      <c r="L3">
-        <v>8</v>
-      </c>
-      <c r="M3">
-        <v>152740</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Dòng ví dụ — xoá trước khi dùng thật</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>HOWO 420</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Lọc nhớt A7</v>
+      </c>
+      <c r="C4" t="str">
         <v>612630010239</v>
       </c>
-      <c r="B4" t="str">
-        <v>JX1016; SMS-10452; CX1020</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Lọc nhớt A7</v>
-      </c>
       <c r="D4" t="str">
-        <v>Oil Filter</v>
+        <v>Normal</v>
       </c>
       <c r="E4" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="F4" t="str">
-        <v>HOWO 420</v>
-      </c>
-      <c r="G4" t="str">
         <v>Cái</v>
       </c>
-      <c r="H4">
+      <c r="F4">
         <v>200</v>
       </c>
-      <c r="I4">
-        <v>87480</v>
-      </c>
-      <c r="J4">
+      <c r="G4">
         <v>3</v>
-      </c>
-      <c r="K4">
-        <v>27000</v>
-      </c>
-      <c r="L4">
-        <v>8</v>
-      </c>
-      <c r="M4">
-        <v>118098</v>
-      </c>
-      <c r="N4" t="str">
-        <v>Ví dụ nhiều mã thay thế cách nhau bằng '; '</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>VD-MINH-HOA</v>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5" t="str">
-        <v>Ví dụ: để trống tỷ giá/VAT/giá bán</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v>SMS</v>
-      </c>
-      <c r="F5" t="str">
-        <v>HOWO 420</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Cái</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5">
-        <v>10</v>
-      </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-      <c r="N5" t="str">
-        <v>Để trống TyGiaUSD/VAT = dùng tỷ giá &amp; VAT trên form (vd 27.000 &amp; 8% → giá vốn 291.600); để trống Giá bán đề xuất = tự tính bằng giá vốn sau VAT + 35% (→ 393.660). Dòng ví dụ — xoá trước khi dùng thật</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A36"/>
   <cols>
     <col min="1" max="1" width="130.83203125" customWidth="1"/>
   </cols>
@@ -667,17 +532,17 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>1. Điền hàng vào sheet 'NhapHang', mỗi dòng = một mặt hàng trong một phiếu nhập. Giữ nguyên hàng tiêu đề (hàng 1).</v>
+        <v>1. Điền hàng vào sheet 'NhapHang', mỗi dòng = một mặt hàng trong một phiếu nhập. Giữ nguyên hàng tiêu đề (hàng 1). Xoá các dòng ví dụ trước khi dùng thật.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Trong app TVK: vào 'Nhập từ Excel', chọn loại phiếu (Nhập mua / Nhập ký gửi), nhà cung cấp, kho, ngày, tỷ giá và VAT mặc định — rồi tải file lên.</v>
+        <v>2. Trong app TVK: vào 'Nhập từ Excel', chọn loại phiếu (Nhập mua / Nhập ký gửi), nhà cung cấp, kho, ngày, rồi nhập Tỷ giá, VAT và % lợi nhuận — rồi tải file lên.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) kèm giá vốn, tỷ giá·VAT áp dụng, thành tiền và giá bán đề xuất — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
+        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) kèm đơn giá nhập VNĐ, thành tiền và giá bán — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
       </c>
     </row>
     <row r="7">
@@ -687,27 +552,27 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GIẢI THÍCH CÁC CỘT</v>
+        <v>GIẢI THÍCH CÁC CỘT (chỉ 7 cột này)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MaHang (BẮT BUỘC): mã chính của phụ tùng (mã OEM). Hệ thống nhận diện hàng theo cột này; trùng mã = nhập thêm vào hàng đã có.</v>
+        <v>DongXe: dòng xe tương thích (vd HOWO 420/430/440) — hệ thống lưu thành dòng xe áp dụng cho hàng.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MaThayThe: các mã tương đương / mã nội bộ (vd mã SMS-xxxxx), cách nhau bằng dấu '; '. Tất cả đều tra cứu và quét mã vạch được.</v>
+        <v>TenHang (BẮT BUỘC): tên phụ tùng. Với hàng mới, tên này thành tên sản phẩm trong danh mục.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TenHang (BẮT BUỘC với hàng mới): tên tiếng Việt. TenTiengAnh: tên tiếng Anh nếu có.</v>
+        <v>MaHang (BẮT BUỘC): mã số của phụ tùng (mã OEM). Hệ thống nhận diện hàng theo cột này; trùng mã = nhập thêm vào hàng đã có.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ThuongHieu: vd SMS, Normal. DongXe: vd HOWO 420 — hệ thống lưu thành dòng xe áp dụng cho hàng.</v>
+        <v>ThuongHieu: vd SMS, Normal — gán cho sản phẩm khi tự tạo mới.</v>
       </c>
     </row>
     <row r="13">
@@ -722,32 +587,32 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GiaVonVND: đơn giá vốn VNĐ (đã gồm VAT nếu có). HOẶC dùng GiaUSD: nếu điền GiaUSD và để trống GiaVonVND,</v>
+        <v>GiaUSD (BẮT BUỘC): đơn giá bằng USD của một đơn vị.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">   hệ thống tự tính Giá vốn = GiaUSD x Tỷ giá x (1 + VAT%) — xem mục CÔNG THỨC bên dưới.</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TyGiaUSD (tuỳ chọn, theo từng dòng): tỷ giá VNĐ/USD riêng của dòng. Để trống = dùng tỷ giá trên form trong app.</v>
+        <v>THÔNG TIN NHẬP TRÊN FORM (áp chung cho toàn bộ file)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>VAT (tuỳ chọn, theo từng dòng, tính theo %): vd 8 = 8%. Để trống = dùng VAT trên form trong app. VAT = 0 nghĩa là không cộng VAT.</v>
+        <v>Tỷ giá (VNĐ/USD): mặc định 27.000 — đổi theo tỷ giá tại thời điểm nhập.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GiaBanDeXuat: giá bán gợi ý — với hàng mới, hệ thống lưu thành giá bán buôn mặc định của sản phẩm. Để trống = tự tính (xem CÔNG THỨC).</v>
+        <v>VAT %: % thuế cộng vào giá USD, mặc định 8%.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GhiChu: ghi chú tự do cho dòng hàng.</v>
+        <v>% lợi nhuận / sản phẩm: mặc định 35% — dùng để tính giá bán.</v>
       </c>
     </row>
     <row r="21">
@@ -757,27 +622,27 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CÔNG THỨC (áp dụng cho mọi dòng)</v>
+        <v>CÔNG THỨC (hệ thống tự tính cho mọi dòng)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>1. Giá vốn một đơn vị = GiaVonVND nếu có; ngược lại = GiaUSD x Tỷ giá x (1 + VAT%).</v>
+        <v>1. Đơn giá nhập VNĐ = GiaUSD x Tỷ giá x (1 + VAT%).</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2. Tỷ giá và VAT lấy theo DÒNG (cột TyGiaUSD / VAT) nếu dòng có ghi; dòng nào để trống thì lấy tỷ giá và VAT trên form trong app (mặc định 27.000 và 8%).</v>
+        <v>2. Thành tiền của dòng = SoLuong x Đơn giá nhập VNĐ.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>3. Thành tiền của dòng = SoLuong x Giá vốn.</v>
+        <v>3. Giá bán = Đơn giá nhập VNĐ x (1 + % lợi nhuận). Với hàng mới, giá bán này thành giá bán sỉ ban đầu của sản phẩm.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>4. Giá bán đề xuất = GiaBanDeXuat nếu có; để trống thì = Giá vốn sau VAT x 1,35 (tức giá vốn + 35%).</v>
+        <v>4. Total giá nhập VND = tổng Thành tiền của tất cả các dòng trong file (hiện ở cuối bảng xem trước).</v>
       </c>
     </row>
     <row r="27">
@@ -787,37 +652,52 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>LƯU Ý</v>
+        <v>VÍ DỤ</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
+        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35% → Đơn giá nhập = 100 x 27.000 x 1,08 = 2.916.000; Giá bán = 2.916.000 x 1,35 = 3.936.600; nhập 15 cái → Thành tiền = 43.740.000.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>- Dòng thiếu MaHang hoặc SoLuong &lt;= 0 sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>- Dòng có TyGiaUSD &lt;= 0 hoặc VAT &lt; 0 cũng bị báo lỗi.</v>
+        <v>LƯU Ý</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm mã thay thế và dòng xe khi bạn xác nhận.</v>
+        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
+        <v>- Dòng thiếu MaHang, TenHang, SoLuong &lt;= 0 hoặc thiếu GiaUSD sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>- Các cột cũ về giá theo dòng (GiaVonVND, TyGiaUSD, VAT, GiaBanDeXuat) không còn dùng — giá và giá bán giờ tính chung từ form.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm dòng xe khi bạn xác nhận.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
         <v>- Chấp nhận file .xlsx và .csv (csv: dùng đúng các tiêu đề cột như trên, mã hoá UTF-8).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Import Excel: correct 8-column format (add TenTiengAnh, accept Vietnamese display headers)
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -398,15 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,18 +418,21 @@
         <v>TenHang</v>
       </c>
       <c r="C1" t="str">
+        <v>TenTiengAnh</v>
+      </c>
+      <c r="D1" t="str">
         <v>MaHang</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>ThuongHieu</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>DonViTinh</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>SoLuong</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>GiaUSD</v>
       </c>
     </row>
@@ -440,18 +444,21 @@
         <v>Bơm nước - 420Hp</v>
       </c>
       <c r="C2" t="str">
+        <v>Water Pump - 420Hp</v>
+      </c>
+      <c r="D2" t="str">
         <v>VG1246060108</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>SMS</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Cái</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>15</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>100</v>
       </c>
     </row>
@@ -463,18 +470,21 @@
         <v>Lọc dầu dưới</v>
       </c>
       <c r="C3" t="str">
+        <v>Fuel Filter</v>
+      </c>
+      <c r="D3" t="str">
         <v>611600080113</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>SMS</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Cái</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>400</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>3.88</v>
       </c>
     </row>
@@ -486,31 +496,34 @@
         <v>Lọc nhớt A7</v>
       </c>
       <c r="C4" t="str">
+        <v>Oil Filter</v>
+      </c>
+      <c r="D4" t="str">
         <v>612630010239</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Normal</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Cái</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>200</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A38"/>
   <cols>
     <col min="1" max="1" width="130.83203125" customWidth="1"/>
   </cols>
@@ -552,152 +565,162 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GIẢI THÍCH CÁC CỘT (chỉ 7 cột này)</v>
+        <v>GIẢI THÍCH CÁC CỘT (chỉ 8 cột này, theo đúng thứ tự)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>DongXe: dòng xe tương thích (vd HOWO 420/430/440) — hệ thống lưu thành dòng xe áp dụng cho hàng.</v>
+        <v>DongXe (Dòng xe): dòng xe tương thích (vd HOWO 420/430/440) — hệ thống lưu thành dòng xe áp dụng cho hàng.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TenHang (BẮT BUỘC): tên phụ tùng. Với hàng mới, tên này thành tên sản phẩm trong danh mục.</v>
+        <v>TenHang (Tên phụ tùng, BẮT BUỘC): tên phụ tùng. Với hàng mới, tên này thành tên sản phẩm trong danh mục.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MaHang (BẮT BUỘC): mã số của phụ tùng (mã OEM). Hệ thống nhận diện hàng theo cột này; trùng mã = nhập thêm vào hàng đã có.</v>
+        <v>TenTiengAnh (Tên tiếng anh): tên tiếng Anh nếu có (không bắt buộc — dòng nào chưa có vẫn nhập được).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ThuongHieu: vd SMS, Normal — gán cho sản phẩm khi tự tạo mới.</v>
+        <v>MaHang (Mã số, BẮT BUỘC): mã số của phụ tùng (mã OEM). Hệ thống nhận diện hàng theo cột này; trùng mã = nhập thêm vào hàng đã có.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>DonViTinh: Cái / Bộ / Chiếc... (mặc định: Cái).</v>
+        <v>ThuongHieu (Thương hiệu): vd SMS, Normal — gán cho sản phẩm khi tự tạo mới.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SoLuong (BẮT BUỘC, &gt; 0).</v>
+        <v>DonViTinh (ĐVT): Cái / Bộ / Chiếc... (mặc định: Cái).</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GiaUSD (BẮT BUỘC): đơn giá bằng USD của một đơn vị.</v>
+        <v>SoLuong (Số lượng, BẮT BUỘC, &gt; 0).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>GiaUSD (Đơn giá USD, BẮT BUỘC): đơn giá bằng USD của một đơn vị.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>THÔNG TIN NHẬP TRÊN FORM (áp chung cho toàn bộ file)</v>
+        <v>Tên cột có thể viết bằng tiếng Việt tương ứng (Dòng xe, Tên phụ tùng, Tên tiếng anh, Mã số, Thương hiệu, ĐVT, Số lượng, Đơn giá USD) — hệ thống vẫn nhận.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Tỷ giá (VNĐ/USD): mặc định 27.000 — đổi theo tỷ giá tại thời điểm nhập.</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>VAT %: % thuế cộng vào giá USD, mặc định 8%.</v>
+        <v>THÔNG TIN NHẬP TRÊN FORM (áp chung cho toàn bộ file)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>% lợi nhuận / sản phẩm: mặc định 35% — dùng để tính giá bán.</v>
+        <v>Tỷ giá (VNĐ/USD): mặc định 27.000 — đổi theo tỷ giá tại thời điểm nhập.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>VAT %: % thuế cộng vào giá USD, mặc định 8%.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>CÔNG THỨC (hệ thống tự tính cho mọi dòng)</v>
+        <v>% lợi nhuận / sản phẩm: mặc định 35% — dùng để tính giá bán.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>1. Đơn giá nhập VNĐ = GiaUSD x Tỷ giá x (1 + VAT%).</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2. Thành tiền của dòng = SoLuong x Đơn giá nhập VNĐ.</v>
+        <v>CÔNG THỨC (hệ thống tự tính cho mọi dòng)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>3. Giá bán = Đơn giá nhập VNĐ x (1 + % lợi nhuận). Với hàng mới, giá bán này thành giá bán sỉ ban đầu của sản phẩm.</v>
+        <v>1. Đơn giá nhập VNĐ = GiaUSD x Tỷ giá x (1 + VAT%).</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>4. Total giá nhập VND = tổng Thành tiền của tất cả các dòng trong file (hiện ở cuối bảng xem trước).</v>
+        <v>2. Thành tiền của dòng = SoLuong x Đơn giá nhập VNĐ.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>3. Giá bán = Đơn giá nhập VNĐ x (1 + % lợi nhuận). Với hàng mới, giá bán này thành giá bán sỉ ban đầu của sản phẩm.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>VÍ DỤ</v>
+        <v>4. Total giá nhập VND = tổng Thành tiền của tất cả các dòng trong file (hiện ở cuối bảng xem trước).</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35% → Đơn giá nhập = 100 x 27.000 x 1,08 = 2.916.000; Giá bán = 2.916.000 x 1,35 = 3.936.600; nhập 15 cái → Thành tiền = 43.740.000.</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
+        <v>VÍ DỤ</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>LƯU Ý</v>
+        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35% → Đơn giá nhập = 100 x 27.000 x 1,08 = 2.916.000; Giá bán = 2.916.000 x 1,35 = 3.936.600; nhập 15 cái → Thành tiền = 43.740.000.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>- Dòng thiếu MaHang, TenHang, SoLuong &lt;= 0 hoặc thiếu GiaUSD sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
+        <v>LƯU Ý</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>- Các cột cũ về giá theo dòng (GiaVonVND, TyGiaUSD, VAT, GiaBanDeXuat) không còn dùng — giá và giá bán giờ tính chung từ form.</v>
+        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm dòng xe khi bạn xác nhận.</v>
+        <v>- Dòng thiếu MaHang, TenHang, SoLuong &lt;= 0 hoặc thiếu GiaUSD sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>- Các cột cũ về giá theo dòng (GiaVonVND, TyGiaUSD, VAT, GiaBanDeXuat) không còn dùng — giá và giá bán giờ tính chung từ form.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm dòng xe khi bạn xác nhận.</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
         <v>- Chấp nhận file .xlsx và .csv (csv: dùng đúng các tiêu đề cột như trên, mã hoá UTF-8).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Display: VND without suffix, USD with $ prefix; import preview adds Don gia USD, renames VND column to Don gia VND + VAT
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -650,17 +650,17 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>1. Đơn giá nhập VNĐ = GiaUSD x Tỷ giá x (1 + VAT%).</v>
+        <v>1. Đơn giá VND + VAT = GiaUSD x Tỷ giá x (1 + VAT%).</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2. Thành tiền của dòng = SoLuong x Đơn giá nhập VNĐ.</v>
+        <v>2. Thành tiền của dòng = SoLuong x Đơn giá VND + VAT.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>3. Giá bán = Đơn giá nhập VNĐ x (1 + % lợi nhuận). Với hàng mới, giá bán này thành giá bán sỉ ban đầu của sản phẩm.</v>
+        <v>3. Giá bán = Đơn giá VND + VAT x (1 + % lợi nhuận). Với hàng mới, giá bán này thành giá bán sỉ ban đầu của sản phẩm.</v>
       </c>
     </row>
     <row r="28">
@@ -680,7 +680,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35% → Đơn giá nhập = 100 x 27.000 x 1,08 = 2.916.000; Giá bán = 2.916.000 x 1,35 = 3.936.600; nhập 15 cái → Thành tiền = 43.740.000.</v>
+        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35% → Đơn giá VND + VAT = 100 x 27.000 x 1,08 = 2.916.000; Giá bán = 2.916.000 x 1,35 = 3.936.600; nhập 15 cái → Thành tiền = 43.740.000.</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
Simplify import footer, remove stock-in explanations, bright 3D sidebar tabs, confirm-now on manual receipts
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -399,16 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H4"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -524,9 +514,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A38"/>
-  <cols>
-    <col min="1" max="1" width="130.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -665,7 +652,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>4. Total giá nhập VND = tổng Thành tiền + Chênh lệch làm tròn (hiện ở cuối bảng xem trước). Chênh lệch làm tròn = làm tròn một lần ở cuối từ giá trị chính xác của từng dòng, trừ đi tổng các dòng (đơn giá đã làm tròn) — nhờ vậy tổng khớp với kế toán trong khi đơn giá từng dòng vẫn khớp hoá đơn nhà cung cấp.</v>
+        <v>4. Total giá nhập VND đã khớp với kế toán: tổng làm tròn một lần ở cuối từ giá trị chính xác của từng dòng (chênh lệch với tổng các dòng được lưu cùng phiếu nhập, không hiện riêng). Đơn giá từng dòng vẫn khớp hoá đơn nhà cung cấp.</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Dealer/retail prices: products columns, import retail pct, sales price basis, light sidebar with footer credit
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -542,7 +542,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) kèm đơn giá nhập VNĐ, thành tiền và giá bán — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
+        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) kèm đơn giá nhập VNĐ, thành tiền, giá đại lý và giá lẻ — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
       </c>
     </row>
     <row r="7">
@@ -622,7 +622,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>% lợi nhuận / sản phẩm: mặc định 35% — dùng để tính giá bán.</v>
+        <v>% lợi nhuận / sản phẩm: mặc định 35% — dùng để tính giá đại lý. % giá bán lẻ: mặc định 50% — dùng để tính giá lẻ.</v>
       </c>
     </row>
     <row r="23">
@@ -647,7 +647,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>3. Giá bán = Đơn giá VND + VAT x (1 + % lợi nhuận). Với hàng mới, giá bán này thành giá bán sỉ ban đầu của sản phẩm.</v>
+        <v>3. Giá đại lý = Đơn giá VND + VAT x (1 + % lợi nhuận); Giá lẻ = Đơn giá VND + VAT x (1 + % giá bán lẻ). Với hàng mới, hai giá này thành giá đại lý và giá lẻ ban đầu của sản phẩm.</v>
       </c>
     </row>
     <row r="28">
@@ -667,7 +667,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35% → Đơn giá VND + VAT = 100 x 27.000 x 1,08 = 2.916.000; Giá bán = 2.916.000 x 1,35 = 3.936.600; nhập 15 cái → Thành tiền = 43.740.000.</v>
+        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35%, Giá lẻ 50% → Đơn giá VND + VAT = 100 x 27.000 x 1,08 = 2.916.000; Giá đại lý = 2.916.000 x 1,35 = 3.936.600; Giá lẻ = 2.916.000 x 1,50 = 4.374.000; nhập 15 cái → Thành tiền = 43.740.000.</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
Them cot HanDung khi import + han dung tren form tay + FEFO cho nhot (migration 0017)
</commit_message>
<xml_diff>
--- a/public/mau-import-nhap-hang.xlsx
+++ b/public/mau-import-nhap-hang.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="NhapHang" sheetId="1" r:id="rId1"/>
-    <sheet name="HuongDan" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,6 +435,9 @@
       <c r="H1" t="str">
         <v>GiaUSD</v>
       </c>
+      <c r="I1" t="str">
+        <v>HanDung</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -451,6 +464,9 @@
       <c r="H2">
         <v>100</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -477,6 +493,9 @@
       <c r="H3">
         <v>3.88</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -503,211 +522,13 @@
       <c r="H4">
         <v>3</v>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A38"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>HƯỚNG DẪN FILE MẪU NHẬP HÀNG — TVK</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>CÁCH DÙNG</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>1. Điền hàng vào sheet 'NhapHang', mỗi dòng = một mặt hàng trong một phiếu nhập. Giữ nguyên hàng tiêu đề (hàng 1). Xoá các dòng ví dụ trước khi dùng thật.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2. Trong app TVK: vào 'Nhập từ Excel', chọn loại phiếu (Nhập mua / Nhập ký gửi), nhà cung cấp, kho, ngày, rồi nhập Tỷ giá, VAT và % lợi nhuận — rồi tải file lên.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>3. Hệ thống xem trước từng dòng (hàng đã có / hàng mới / lỗi) kèm đơn giá nhập VNĐ, thành tiền, giá đại lý và giá lẻ — kiểm tra rồi bấm Xác nhận để tạo phiếu nhập.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>GIẢI THÍCH CÁC CỘT (chỉ 8 cột này, theo đúng thứ tự)</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>DongXe (Dòng xe): dòng xe tương thích (vd HOWO 420/430/440) — hệ thống lưu thành dòng xe áp dụng cho hàng.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>TenHang (Tên phụ tùng, BẮT BUỘC): tên phụ tùng. Với hàng mới, tên này thành tên sản phẩm trong danh mục.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>TenTiengAnh (Tên tiếng anh): tên tiếng Anh nếu có (không bắt buộc — dòng nào chưa có vẫn nhập được).</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>MaHang (Mã số, BẮT BUỘC): mã số của phụ tùng (mã OEM). Hệ thống nhận diện hàng theo cột này; trùng mã = nhập thêm vào hàng đã có.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>ThuongHieu (Thương hiệu): vd SMS, Normal — gán cho sản phẩm khi tự tạo mới.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>DonViTinh (ĐVT): Cái / Bộ / Chiếc... (mặc định: Cái).</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>SoLuong (Số lượng, BẮT BUỘC, &gt; 0).</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>GiaUSD (Đơn giá USD, BẮT BUỘC): đơn giá bằng USD của một đơn vị.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Tên cột có thể viết bằng tiếng Việt tương ứng (Dòng xe, Tên phụ tùng, Tên tiếng anh, Mã số, Thương hiệu, ĐVT, Số lượng, Đơn giá USD) — hệ thống vẫn nhận.</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>THÔNG TIN NHẬP TRÊN FORM (áp chung cho toàn bộ file)</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Tỷ giá (VNĐ/USD): mặc định 27.000 — đổi theo tỷ giá tại thời điểm nhập.</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>VAT %: % thuế cộng vào giá USD, mặc định 8%.</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>% lợi nhuận / sản phẩm: mặc định 35% — dùng để tính giá đại lý. % giá bán lẻ: mặc định 50% — dùng để tính giá lẻ.</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>CÔNG THỨC (hệ thống tự tính cho mọi dòng)</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>1. Đơn giá VND + VAT = GiaUSD x Tỷ giá x (1 + VAT%).</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>2. Thành tiền của dòng = SoLuong x Đơn giá VND + VAT.</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>3. Giá đại lý = Đơn giá VND + VAT x (1 + % lợi nhuận); Giá lẻ = Đơn giá VND + VAT x (1 + % giá bán lẻ). Với hàng mới, hai giá này thành giá đại lý và giá lẻ ban đầu của sản phẩm.</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>4. Total giá nhập VND đã khớp với kế toán: tổng làm tròn một lần ở cuối từ giá trị chính xác của từng dòng (chênh lệch với tổng các dòng được lưu cùng phiếu nhập, không hiện riêng). Đơn giá từng dòng vẫn khớp hoá đơn nhà cung cấp.</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>VÍ DỤ</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>GiaUSD 100, Tỷ giá 27.000, VAT 8%, Lợi nhuận 35%, Giá lẻ 50% → Đơn giá VND + VAT = 100 x 27.000 x 1,08 = 2.916.000; Giá đại lý = 2.916.000 x 1,35 = 3.936.600; Giá lẻ = 2.916.000 x 1,50 = 4.374.000; nhập 15 cái → Thành tiền = 43.740.000.</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>LƯU Ý</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>- Một file = một phiếu nhập của MỘT nhà cung cấp (chọn nhà cung cấp trên form trong app, không điền trong file).</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>- Dòng thiếu MaHang, TenHang, SoLuong &lt;= 0 hoặc thiếu GiaUSD sẽ bị báo lỗi ở màn hình xem trước và không được nhập.</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>- Các cột cũ về giá theo dòng (GiaVonVND, TyGiaUSD, VAT, GiaBanDeXuat) không còn dùng — giá và giá bán giờ tính chung từ form.</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>- Hàng mới (mã chưa có trong hệ thống) sẽ được tự tạo kèm dòng xe khi bạn xác nhận.</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>- Chấp nhận file .xlsx và .csv (csv: dùng đúng các tiêu đề cột như trên, mã hoá UTF-8).</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>